<commit_message>
refactor: base de datos de pacientes sólo para primera sesión presencial (excluye llamadas), sin estado y formato exclusivo xlsx
</commit_message>
<xml_diff>
--- a/docs/pacientes_primera_sesion.xlsx
+++ b/docs/pacientes_primera_sesion.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -467,9 +467,6 @@
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -498,21 +495,6 @@
           <t>Motivo de Consulta</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Tipo de Cita</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Fecha de Registro</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -540,21 +522,6 @@
           <t>RPG y terapias manuales</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Agendado</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -582,21 +549,6 @@
           <t>Rehabilitación de hombro</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Agendado</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -624,21 +576,6 @@
           <t>Reeducación postural</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Agendado</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -666,21 +603,6 @@
           <t>Dolor articular y movilidad</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Agendado</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
-        </is>
-      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -708,21 +630,6 @@
           <t>Cervicalgia y tensión escapular</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Agendado</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
-        </is>
-      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -750,26 +657,11 @@
           <t>Dolor de espalda / Traumatología</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Agendado</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lic. Norberto Brude</t>
+          <t>Mariana González Cadahia</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -779,7 +671,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>+54 9 11 6156-4311</t>
+          <t>+54 9 11 4455-6677</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -789,29 +681,14 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>ATM / Bruxismo y dolor mandibular</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Llamada de Orientación (15m)</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Confirmado</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
+          <t>Reeducación Postural Global (RPG) / Columna</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Mariana González Cadahia</t>
+          <t>Sofía Finocchio Gonzalez</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -821,39 +698,24 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+54 9 11 4455-6677</t>
+          <t>+54 9 11 3322-1100</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>2026-09-30 10:00</t>
+          <t>2026-09-30 08:45</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Reeducación Postural Global (RPG) / Columna</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Confirmado</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
+          <t>ATM y contractura cervical</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Sofía Finocchio Gonzalez</t>
+          <t>Alejandro Wainschenker</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -863,39 +725,24 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>+54 9 11 3322-1100</t>
+          <t>+54 9 11 3344-5566</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30 08:45</t>
+          <t>2026-09-29 18:00</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>ATM y contractura cervical</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Agendado</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
+          <t>Rehabilitación motora</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Alejandro Wainschenker</t>
+          <t>Constancia Tiboni</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -905,116 +752,44 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+54 9 11 3344-5566</t>
+          <t>+54 9 11 5566-7788</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29 18:00</t>
+          <t>2026-09-29 16:00</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Rehabilitación motora</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Realizado</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
+          <t>Evaluación postural y dolor cervical</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Constancia Tiboni</t>
+          <t>Lucas Méndez</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>No provisto</t>
+          <t>38123456</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+54 9 11 5566-7788</t>
+          <t>+54 9 11 4455-6677</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2026-09-29 16:00</t>
+          <t>2026-09-28 16:00</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Evaluación postural y dolor cervical</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Realizado</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Lucas Méndez</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>38123456</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>+54 9 11 4455-6677</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-28 16:00</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
           <t>Lumbalgia aguda y postura</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Turno Presencial (1h)</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Confirmado</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-29 23:08:56</t>
         </is>
       </c>
     </row>

</xml_diff>